<commit_message>
code_book(): the Excel workbook reviewed, `position` in values, the running head echoes the cover
Excel: the notes wrap in a wide Value column; in `variables` the
position, name and label stay in view; every sheet prints in landscape
fitted to the page width with its header row repeated; the mean, SD and
median carry a number format at the precision of the PDF, and the
column widths come from the numbers as displayed. The columns are always
the same, empty when they do not apply. `values` gains `position`, in
the object and in the workbook. The running head of the PDF sets the
word Codebook in spaced capitals, as the cover does. The cover takes the
width of the README.
</commit_message>
<xml_diff>
--- a/pkgdown/assets/codebook/sochealth_codebook.xlsx
+++ b/pkgdown/assets/codebook/sochealth_codebook.xlsx
@@ -10,13 +10,28 @@
     <sheet name="variables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="values" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName localSheetId="0" name="_xlnm.Print_Titles">'codebook'!$1:$1</definedName>
+    <definedName localSheetId="1" name="_xlnm.Print_Titles">'variables'!$1:$1</definedName>
+    <definedName localSheetId="2" name="_xlnm.Print_Titles">'values'!$1:$1</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
+  <numFmts count="11">
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="0.00"/>
+    <numFmt numFmtId="170" formatCode="0.00"/>
+    <numFmt numFmtId="171" formatCode="0.00"/>
+    <numFmt numFmtId="172" formatCode="0.00"/>
+    <numFmt numFmtId="173" formatCode="0.00"/>
+    <numFmt numFmtId="174" formatCode="0.00"/>
+    <numFmt numFmtId="175" formatCode="0.000"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,11 +73,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf applyFill="1" borderId="0" fillId="2" fontId="0" numFmtId="0" xfId="0"/>
     <xf applyFill="1" applyFont="1" borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="165" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="166" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="167" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="168" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="169" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="170" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="171" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="172" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="173" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="174" xfId="0"/>
+    <xf applyNumberFormat="1" borderId="0" fillId="0" fontId="0" numFmtId="175" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,11 +416,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="16.711"/>
-    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="60.711"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="90.711"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -408,191 +439,194 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Social health survey</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Subtitle</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Simulated data shipped with spicy</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Jane Doe – University of Somewhere – ORCID 0000-0002-1825-0097</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>John Doe – Somewhere Institute of Public Health</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>1200</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Variables</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>24</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Counts and percentages are unweighted: they describe the data file and are not estimates for a population.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Simulated data shipped with spicy (?sochealth): 1,200 respondents of a fictitious social health survey, built to document the package. Nothing here describes a real population.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Source and citation: https://amaltawfik.github.io/spicy/ and doi:10.32614/CRAN.package.spicy.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>- weight is the survey design weight (0.29 to 3.45): the counts of this codebook are unweighted.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>- bmi is in kg/m2, and bmi_category follows it (normal weight, overweight, obesity).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>- The four life_sat_* items run from 1 to 5 (Likert scale).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>- response_date is the time of the interview, Europe/Zurich.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Generated with</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>spicy 0.13.0.9000, R 4.6.1, 2026-10-09 18:29:22</t>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>spicy 0.13.0.9000, R 4.6.1, 2026-10-09 18:53:15</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
-  <printOptions gridLines="1" gridLinesSet="1"/>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" fitToHeight="0" fitToWidth="1" scale="100"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -607,10 +641,7 @@
     <col min="10" max="10" bestFit="1" customWidth="1" hidden="false" width="24.711"/>
     <col min="11" max="11" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
     <col min="12" max="12" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
-    <col min="13" max="14" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
-    <col min="15" max="15" bestFit="1" customWidth="1" hidden="false" width="19.711"/>
-    <col min="16" max="16" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
-    <col min="17" max="17" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
+    <col min="13" max="17" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
     <col min="18" max="19" bestFit="1" customWidth="1" hidden="false" width="35.711"/>
   </cols>
   <sheetData>
@@ -803,13 +834,13 @@
       <c r="N3">
         <v>75</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="5">
         <v>49.2641666666667</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="5">
         <v>14.7042928934649</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="5">
         <v>48.5</v>
       </c>
     </row>
@@ -1130,13 +1161,13 @@
       <c r="N10">
         <v>7388</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="6">
         <v>3832.99583333333</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="6">
         <v>1394.58423857484</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="6">
         <v>3784</v>
       </c>
     </row>
@@ -1367,13 +1398,13 @@
       <c r="N15">
         <v>100</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="7">
         <v>69.0405833333333</v>
       </c>
-      <c r="P15">
+      <c r="P15" s="7">
         <v>15.6203587559989</v>
       </c>
-      <c r="Q15">
+      <c r="Q15" s="7">
         <v>70.25</v>
       </c>
     </row>
@@ -1424,13 +1455,13 @@
       <c r="N16">
         <v>38.9</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="8">
         <v>25.9314814814815</v>
       </c>
-      <c r="P16">
+      <c r="P16" s="8">
         <v>3.72018590188177</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="8">
         <v>25.9</v>
       </c>
     </row>
@@ -1571,13 +1602,13 @@
       <c r="N19">
         <v>10</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="9">
         <v>5.48016877637131</v>
       </c>
-      <c r="P19">
+      <c r="P19" s="9">
         <v>2.03387361047396</v>
       </c>
-      <c r="Q19">
+      <c r="Q19" s="9">
         <v>6</v>
       </c>
     </row>
@@ -1628,13 +1659,13 @@
       <c r="N20">
         <v>5</v>
       </c>
-      <c r="O20">
+      <c r="O20" s="10">
         <v>3.54865771812081</v>
       </c>
-      <c r="P20">
+      <c r="P20" s="10">
         <v>1.25008072026489</v>
       </c>
-      <c r="Q20">
+      <c r="Q20" s="10">
         <v>4</v>
       </c>
     </row>
@@ -1685,13 +1716,13 @@
       <c r="N21">
         <v>5</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="11">
         <v>3.37835570469799</v>
       </c>
-      <c r="P21">
+      <c r="P21" s="11">
         <v>1.18497505958556</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="11">
         <v>3</v>
       </c>
     </row>
@@ -1742,13 +1773,13 @@
       <c r="N22">
         <v>5</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="12">
         <v>3.7248322147651</v>
       </c>
-      <c r="P22">
+      <c r="P22" s="12">
         <v>1.09718553250181</v>
       </c>
-      <c r="Q22">
+      <c r="Q22" s="12">
         <v>4</v>
       </c>
     </row>
@@ -1799,13 +1830,13 @@
       <c r="N23">
         <v>5</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="13">
         <v>3.39681208053691</v>
       </c>
-      <c r="P23">
+      <c r="P23" s="13">
         <v>1.16025268893811</v>
       </c>
-      <c r="Q23">
+      <c r="Q23" s="13">
         <v>4</v>
       </c>
     </row>
@@ -1908,1246 +1939,1402 @@
       <c r="N25">
         <v>3.447</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="14">
         <v>0.997061666666667</v>
       </c>
-      <c r="P25">
+      <c r="P25" s="14">
         <v>0.40625697754877</v>
       </c>
-      <c r="Q25">
+      <c r="Q25" s="14">
         <v>0.913</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
-  <printOptions gridLines="1" gridLinesSet="1"/>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" fitToHeight="0" fitToWidth="1" scale="100"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:G50"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="21.711"/>
-    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
-    <col min="3" max="3" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
-    <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
-    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
-    <col min="6" max="7" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="21.711"/>
+    <col min="3" max="3" bestFit="1" customWidth="1" hidden="false" width="17.711"/>
+    <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
+    <col min="5" max="5" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
+    <col min="6" max="7" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
+    <col min="8" max="8" bestFit="1" customWidth="1" hidden="false" width="9.711"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>Pos.</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Declared missing</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Valid %</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="D2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2">
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>620</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="4">
         <v>51.6666666666667</v>
       </c>
-      <c r="G2" s="3">
+      <c r="H2" s="4">
         <v>51.6666666666667</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="D3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E3">
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3">
         <v>580</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="4">
         <v>48.3333333333333</v>
       </c>
-      <c r="G3" s="3">
+      <c r="H3" s="4">
         <v>48.3333333333333</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>age_group</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>25-34</t>
         </is>
       </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4">
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>242</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="4">
         <v>20.1666666666667</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="4">
         <v>20.1666666666667</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>age_group</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>35-49</t>
         </is>
       </c>
-      <c r="D5" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>383</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="4">
         <v>31.9166666666667</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="4">
         <v>31.9166666666667</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>age_group</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>50-64</t>
         </is>
       </c>
-      <c r="D6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6">
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6">
         <v>327</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="4">
         <v>27.25</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="4">
         <v>27.25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>age_group</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>65-75</t>
         </is>
       </c>
-      <c r="D7" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7">
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7">
         <v>248</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="4">
         <v>20.6666666666667</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="4">
         <v>20.6666666666667</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>education</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Lower secondary</t>
         </is>
       </c>
-      <c r="D8" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8">
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8">
         <v>261</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="4">
         <v>21.75</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="4">
         <v>21.75</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>education</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Upper secondary</t>
         </is>
       </c>
-      <c r="D9" t="b">
-        <v>0</v>
-      </c>
-      <c r="E9">
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9">
         <v>539</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="4">
         <v>44.9166666666667</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="4">
         <v>44.9166666666667</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>education</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Tertiary</t>
         </is>
       </c>
-      <c r="D10" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10">
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10">
         <v>400</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="4">
         <v>33.3333333333333</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H10" s="4">
         <v>33.3333333333333</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>social_class</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Lower</t>
         </is>
       </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11">
+      <c r="E11" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11">
         <v>144</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="4">
         <v>12</v>
       </c>
-      <c r="G11" s="3">
+      <c r="H11" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>social_class</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Working</t>
         </is>
       </c>
-      <c r="D12" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12">
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12">
         <v>278</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="4">
         <v>23.1666666666667</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="4">
         <v>23.1666666666667</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>social_class</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Lower middle</t>
         </is>
       </c>
-      <c r="D13" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13">
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13">
         <v>326</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G13" s="4">
         <v>27.1666666666667</v>
       </c>
-      <c r="G13" s="3">
+      <c r="H13" s="4">
         <v>27.1666666666667</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>social_class</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Middle</t>
         </is>
       </c>
-      <c r="D14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14">
+      <c r="E14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14">
         <v>306</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="4">
         <v>25.5</v>
       </c>
-      <c r="G14" s="3">
+      <c r="H14" s="4">
         <v>25.5</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>social_class</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Upper middle</t>
         </is>
       </c>
-      <c r="D15" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15">
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15">
         <v>146</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G15" s="4">
         <v>12.1666666666667</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H15" s="4">
         <v>12.1666666666667</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="D16" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16">
+      <c r="E16" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16">
         <v>245</v>
       </c>
-      <c r="F16" s="3">
+      <c r="G16" s="4">
         <v>20.4166666666667</v>
       </c>
-      <c r="G16" s="3">
+      <c r="H16" s="4">
         <v>20.4166666666667</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17">
+        <v>6</v>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>East</t>
         </is>
       </c>
-      <c r="D17" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17">
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17">
         <v>145</v>
       </c>
-      <c r="F17" s="3">
+      <c r="G17" s="4">
         <v>12.0833333333333</v>
       </c>
-      <c r="G17" s="3">
+      <c r="H17" s="4">
         <v>12.0833333333333</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>North</t>
         </is>
       </c>
-      <c r="D18" t="b">
-        <v>0</v>
-      </c>
-      <c r="E18">
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18">
         <v>203</v>
       </c>
-      <c r="F18" s="3">
+      <c r="G18" s="4">
         <v>16.9166666666667</v>
       </c>
-      <c r="G18" s="3">
+      <c r="H18" s="4">
         <v>16.9166666666667</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="D19" t="b">
-        <v>0</v>
-      </c>
-      <c r="E19">
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19">
         <v>198</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="4">
         <v>16.5</v>
       </c>
-      <c r="G19" s="3">
+      <c r="H19" s="4">
         <v>16.5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>South</t>
         </is>
       </c>
-      <c r="D20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E20">
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20">
         <v>201</v>
       </c>
-      <c r="F20" s="3">
+      <c r="G20" s="4">
         <v>16.75</v>
       </c>
-      <c r="G20" s="3">
+      <c r="H20" s="4">
         <v>16.75</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21">
+        <v>6</v>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="D21" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21">
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21">
         <v>208</v>
       </c>
-      <c r="F21" s="3">
+      <c r="G21" s="4">
         <v>17.3333333333333</v>
       </c>
-      <c r="G21" s="3">
+      <c r="H21" s="4">
         <v>17.3333333333333</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22">
+        <v>7</v>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>employment_status</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Employed</t>
         </is>
       </c>
-      <c r="D22" t="b">
-        <v>0</v>
-      </c>
-      <c r="E22">
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22">
         <v>762</v>
       </c>
-      <c r="F22" s="3">
+      <c r="G22" s="4">
         <v>63.5</v>
       </c>
-      <c r="G22" s="3">
+      <c r="H22" s="4">
         <v>63.5</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23">
+        <v>7</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>employment_status</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Student</t>
         </is>
       </c>
-      <c r="D23" t="b">
-        <v>0</v>
-      </c>
-      <c r="E23">
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23">
         <v>143</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="4">
         <v>11.9166666666667</v>
       </c>
-      <c r="G23" s="3">
+      <c r="H23" s="4">
         <v>11.9166666666667</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>employment_status</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Unemployed</t>
         </is>
       </c>
-      <c r="D24" t="b">
-        <v>0</v>
-      </c>
-      <c r="E24">
+      <c r="E24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24">
         <v>174</v>
       </c>
-      <c r="F24" s="3">
+      <c r="G24" s="4">
         <v>14.5</v>
       </c>
-      <c r="G24" s="3">
+      <c r="H24" s="4">
         <v>14.5</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25">
+        <v>7</v>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>employment_status</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="D25" t="b">
-        <v>0</v>
-      </c>
-      <c r="E25">
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25">
         <v>121</v>
       </c>
-      <c r="F25" s="3">
+      <c r="G25" s="4">
         <v>10.0833333333333</v>
       </c>
-      <c r="G25" s="3">
+      <c r="H25" s="4">
         <v>10.0833333333333</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26">
+        <v>8</v>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>income_group</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D26" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26">
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26">
         <v>247</v>
       </c>
-      <c r="F26" s="3">
+      <c r="G26" s="4">
         <v>20.5833333333333</v>
       </c>
-      <c r="G26" s="3">
+      <c r="H26" s="4">
         <v>20.8967851099831</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27">
+        <v>8</v>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>income_group</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Lower middle</t>
         </is>
       </c>
-      <c r="D27" t="b">
-        <v>0</v>
-      </c>
-      <c r="E27">
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27">
         <v>388</v>
       </c>
-      <c r="F27" s="3">
+      <c r="G27" s="4">
         <v>32.3333333333333</v>
       </c>
-      <c r="G27" s="3">
+      <c r="H27" s="4">
         <v>32.8257191201354</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28">
+        <v>8</v>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>income_group</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Upper middle</t>
         </is>
       </c>
-      <c r="D28" t="b">
-        <v>0</v>
-      </c>
-      <c r="E28">
+      <c r="E28" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28">
         <v>328</v>
       </c>
-      <c r="F28" s="3">
+      <c r="G28" s="4">
         <v>27.3333333333333</v>
       </c>
-      <c r="G28" s="3">
+      <c r="H28" s="4">
         <v>27.7495769881557</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29">
+        <v>8</v>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>income_group</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D29" t="b">
-        <v>0</v>
-      </c>
-      <c r="E29">
+      <c r="E29" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29">
         <v>219</v>
       </c>
-      <c r="F29" s="3">
+      <c r="G29" s="4">
         <v>18.25</v>
       </c>
-      <c r="G29" s="3">
+      <c r="H29" s="4">
         <v>18.5279187817259</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30">
+        <v>8</v>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>income_group</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="D30" t="b">
-        <v>0</v>
-      </c>
-      <c r="E30">
+      <c r="E30" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30">
         <v>18</v>
       </c>
-      <c r="F30" s="3">
+      <c r="G30" s="4">
         <v>1.5</v>
       </c>
-      <c r="G30" s="3"/>
+      <c r="H30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31">
+        <v>10</v>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>smoking</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D31" t="b">
-        <v>0</v>
-      </c>
-      <c r="E31">
+      <c r="E31" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31">
         <v>926</v>
       </c>
-      <c r="F31" s="3">
+      <c r="G31" s="4">
         <v>77.1666666666667</v>
       </c>
-      <c r="G31" s="3">
+      <c r="H31" s="4">
         <v>78.8085106382979</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32">
+        <v>10</v>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>smoking</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D32" t="b">
-        <v>0</v>
-      </c>
-      <c r="E32">
+      <c r="E32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32">
         <v>249</v>
       </c>
-      <c r="F32" s="3">
+      <c r="G32" s="4">
         <v>20.75</v>
       </c>
-      <c r="G32" s="3">
+      <c r="H32" s="4">
         <v>21.1914893617021</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33">
+        <v>10</v>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>smoking</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="D33" t="b">
-        <v>0</v>
-      </c>
-      <c r="E33">
+      <c r="E33" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33">
         <v>25</v>
       </c>
-      <c r="F33" s="3">
+      <c r="G33" s="4">
         <v>2.08333333333333</v>
       </c>
-      <c r="G33" s="3"/>
+      <c r="H33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34">
+        <v>11</v>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>physical_activity</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D34" t="b">
-        <v>0</v>
-      </c>
-      <c r="E34">
+      <c r="E34" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34">
         <v>650</v>
       </c>
-      <c r="F34" s="3">
+      <c r="G34" s="4">
         <v>54.1666666666667</v>
       </c>
-      <c r="G34" s="3">
+      <c r="H34" s="4">
         <v>54.1666666666667</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35">
+        <v>11</v>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>physical_activity</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D35" t="b">
-        <v>0</v>
-      </c>
-      <c r="E35">
+      <c r="E35" t="b">
+        <v>0</v>
+      </c>
+      <c r="F35">
         <v>550</v>
       </c>
-      <c r="F35" s="3">
+      <c r="G35" s="4">
         <v>45.8333333333333</v>
       </c>
-      <c r="G35" s="3">
+      <c r="H35" s="4">
         <v>45.8333333333333</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36">
+        <v>12</v>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>dentist_12m</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D36" t="b">
-        <v>0</v>
-      </c>
-      <c r="E36">
+      <c r="E36" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36">
         <v>354</v>
       </c>
-      <c r="F36" s="3">
+      <c r="G36" s="4">
         <v>29.5</v>
       </c>
-      <c r="G36" s="3">
+      <c r="H36" s="4">
         <v>29.5</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37">
+        <v>12</v>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>dentist_12m</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D37" t="b">
-        <v>0</v>
-      </c>
-      <c r="E37">
+      <c r="E37" t="b">
+        <v>0</v>
+      </c>
+      <c r="F37">
         <v>846</v>
       </c>
-      <c r="F37" s="3">
+      <c r="G37" s="4">
         <v>70.5</v>
       </c>
-      <c r="G37" s="3">
+      <c r="H37" s="4">
         <v>70.5</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38">
+        <v>13</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>self_rated_health</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Poor</t>
         </is>
       </c>
-      <c r="D38" t="b">
-        <v>0</v>
-      </c>
-      <c r="E38">
+      <c r="E38" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38">
         <v>61</v>
       </c>
-      <c r="F38" s="3">
+      <c r="G38" s="4">
         <v>5.08333333333333</v>
       </c>
-      <c r="G38" s="3">
+      <c r="H38" s="4">
         <v>5.16949152542373</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39">
+        <v>13</v>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>self_rated_health</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="D39" t="b">
-        <v>0</v>
-      </c>
-      <c r="E39">
+      <c r="E39" t="b">
+        <v>0</v>
+      </c>
+      <c r="F39">
         <v>266</v>
       </c>
-      <c r="F39" s="3">
+      <c r="G39" s="4">
         <v>22.1666666666667</v>
       </c>
-      <c r="G39" s="3">
+      <c r="H39" s="4">
         <v>22.5423728813559</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40">
+        <v>13</v>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>self_rated_health</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="D40" t="b">
-        <v>0</v>
-      </c>
-      <c r="E40">
+      <c r="E40" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40">
         <v>558</v>
       </c>
-      <c r="F40" s="3">
+      <c r="G40" s="4">
         <v>46.5</v>
       </c>
-      <c r="G40" s="3">
+      <c r="H40" s="4">
         <v>47.2881355932203</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41">
+        <v>13</v>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>self_rated_health</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Very good</t>
         </is>
       </c>
-      <c r="D41" t="b">
-        <v>0</v>
-      </c>
-      <c r="E41">
+      <c r="E41" t="b">
+        <v>0</v>
+      </c>
+      <c r="F41">
         <v>295</v>
       </c>
-      <c r="F41" s="3">
+      <c r="G41" s="4">
         <v>24.5833333333333</v>
       </c>
-      <c r="G41" s="3">
+      <c r="H41" s="4">
         <v>25</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42">
+        <v>13</v>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>self_rated_health</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="D42" t="b">
-        <v>0</v>
-      </c>
-      <c r="E42">
+      <c r="E42" t="b">
+        <v>0</v>
+      </c>
+      <c r="F42">
         <v>20</v>
       </c>
-      <c r="F42" s="3">
+      <c r="G42" s="4">
         <v>1.66666666666667</v>
       </c>
-      <c r="G42" s="3"/>
+      <c r="H42" s="4"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43">
+        <v>16</v>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>bmi_category</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Normal weight</t>
         </is>
       </c>
-      <c r="D43" t="b">
-        <v>0</v>
-      </c>
-      <c r="E43">
+      <c r="E43" t="b">
+        <v>0</v>
+      </c>
+      <c r="F43">
         <v>465</v>
       </c>
-      <c r="F43" s="3">
+      <c r="G43" s="4">
         <v>38.75</v>
       </c>
-      <c r="G43" s="3">
+      <c r="H43" s="4">
         <v>39.1414141414141</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44">
+        <v>16</v>
+      </c>
+      <c r="B44" t="inlineStr">
         <is>
           <t>bmi_category</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Overweight</t>
         </is>
       </c>
-      <c r="D44" t="b">
-        <v>0</v>
-      </c>
-      <c r="E44">
+      <c r="E44" t="b">
+        <v>0</v>
+      </c>
+      <c r="F44">
         <v>569</v>
       </c>
-      <c r="F44" s="3">
+      <c r="G44" s="4">
         <v>47.4166666666667</v>
       </c>
-      <c r="G44" s="3">
+      <c r="H44" s="4">
         <v>47.8956228956229</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45">
+        <v>16</v>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>bmi_category</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Obesity</t>
         </is>
       </c>
-      <c r="D45" t="b">
-        <v>0</v>
-      </c>
-      <c r="E45">
+      <c r="E45" t="b">
+        <v>0</v>
+      </c>
+      <c r="F45">
         <v>154</v>
       </c>
-      <c r="F45" s="3">
+      <c r="G45" s="4">
         <v>12.8333333333333</v>
       </c>
-      <c r="G45" s="3">
+      <c r="H45" s="4">
         <v>12.962962962963</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46">
+        <v>16</v>
+      </c>
+      <c r="B46" t="inlineStr">
         <is>
           <t>bmi_category</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="D46" t="b">
-        <v>0</v>
-      </c>
-      <c r="E46">
+      <c r="E46" t="b">
+        <v>0</v>
+      </c>
+      <c r="F46">
         <v>12</v>
       </c>
-      <c r="F46" s="3">
+      <c r="G46" s="4">
         <v>1</v>
       </c>
-      <c r="G46" s="3"/>
+      <c r="H46" s="4"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47">
+        <v>17</v>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>institutional_trust</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Very low</t>
         </is>
       </c>
-      <c r="D47" t="b">
-        <v>0</v>
-      </c>
-      <c r="E47">
+      <c r="E47" t="b">
+        <v>0</v>
+      </c>
+      <c r="F47">
         <v>366</v>
       </c>
-      <c r="F47" s="3">
+      <c r="G47" s="4">
         <v>30.5</v>
       </c>
-      <c r="G47" s="3">
+      <c r="H47" s="4">
         <v>30.5</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48">
+        <v>17</v>
+      </c>
+      <c r="B48" t="inlineStr">
         <is>
           <t>institutional_trust</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D48" t="b">
-        <v>0</v>
-      </c>
-      <c r="E48">
+      <c r="E48" t="b">
+        <v>0</v>
+      </c>
+      <c r="F48">
         <v>472</v>
       </c>
-      <c r="F48" s="3">
+      <c r="G48" s="4">
         <v>39.3333333333333</v>
       </c>
-      <c r="G48" s="3">
+      <c r="H48" s="4">
         <v>39.3333333333333</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49">
+        <v>17</v>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>institutional_trust</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D49" t="b">
-        <v>0</v>
-      </c>
-      <c r="E49">
+      <c r="E49" t="b">
+        <v>0</v>
+      </c>
+      <c r="F49">
         <v>234</v>
       </c>
-      <c r="F49" s="3">
+      <c r="G49" s="4">
         <v>19.5</v>
       </c>
-      <c r="G49" s="3">
+      <c r="H49" s="4">
         <v>19.5</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50">
+        <v>17</v>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>institutional_trust</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Very high</t>
         </is>
       </c>
-      <c r="D50" t="b">
-        <v>0</v>
-      </c>
-      <c r="E50">
+      <c r="E50" t="b">
+        <v>0</v>
+      </c>
+      <c r="F50">
         <v>128</v>
       </c>
-      <c r="F50" s="3">
+      <c r="G50" s="4">
         <v>10.6666666666667</v>
       </c>
-      <c r="G50" s="3">
+      <c r="H50" s="4">
         <v>10.6666666666667</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
-  <printOptions gridLines="1" gridLinesSet="1"/>
+  <autoFilter ref="A1:H1"/>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" fitToHeight="0" fitToWidth="1" scale="100"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Showcase: no invented source codes; sochealth has none
</commit_message>
<xml_diff>
--- a/pkgdown/assets/codebook/sochealth_codebook.xlsx
+++ b/pkgdown/assets/codebook/sochealth_codebook.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>spicy 0.13.0.9000, R 4.6.1, 2026-10-09 18:53:15</t>
+          <t>spicy 0.13.0.9000, R 4.6.1, 2026-10-09 19:18:00</t>
         </is>
       </c>
     </row>
@@ -766,11 +766,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
       <c r="G2">
         <v>1200</v>
       </c>
@@ -811,11 +806,6 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
       <c r="G3">
         <v>1200</v>
       </c>
@@ -868,11 +858,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
       <c r="G4">
         <v>1200</v>
       </c>
@@ -913,11 +898,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
       <c r="G5">
         <v>1200</v>
       </c>
@@ -958,11 +938,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Q5</t>
-        </is>
-      </c>
       <c r="G6">
         <v>1200</v>
       </c>
@@ -1003,11 +978,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
       <c r="G7">
         <v>1200</v>
       </c>
@@ -1048,11 +1018,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Q7</t>
-        </is>
-      </c>
       <c r="G8">
         <v>1200</v>
       </c>
@@ -1093,11 +1058,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Q8</t>
-        </is>
-      </c>
       <c r="G9">
         <v>1182</v>
       </c>
@@ -1138,11 +1098,6 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Q9</t>
-        </is>
-      </c>
       <c r="G10">
         <v>1200</v>
       </c>
@@ -1195,11 +1150,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
       <c r="G11">
         <v>1175</v>
       </c>
@@ -1240,11 +1190,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
       <c r="G12">
         <v>1200</v>
       </c>
@@ -1285,11 +1230,6 @@
           <t>factor</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
       <c r="G13">
         <v>1200</v>
       </c>
@@ -1330,11 +1270,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
       <c r="G14">
         <v>1180</v>
       </c>
@@ -1375,11 +1310,6 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Q14</t>
-        </is>
-      </c>
       <c r="G15">
         <v>1200</v>
       </c>
@@ -1432,11 +1362,6 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Q15</t>
-        </is>
-      </c>
       <c r="G16">
         <v>1188</v>
       </c>
@@ -1489,11 +1414,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Q16</t>
-        </is>
-      </c>
       <c r="G17">
         <v>1188</v>
       </c>
@@ -1534,11 +1454,6 @@
           <t>ordered, factor</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Q17</t>
-        </is>
-      </c>
       <c r="G18">
         <v>1200</v>
       </c>
@@ -1579,11 +1494,6 @@
           <t>numeric</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Q18</t>
-        </is>
-      </c>
       <c r="G19">
         <v>1185</v>
       </c>
@@ -1636,11 +1546,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
       <c r="G20">
         <v>1192</v>
       </c>
@@ -1693,11 +1598,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Q20</t>
-        </is>
-      </c>
       <c r="G21">
         <v>1192</v>
       </c>
@@ -1750,11 +1650,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Q21</t>
-        </is>
-      </c>
       <c r="G22">
         <v>1192</v>
       </c>
@@ -1807,11 +1702,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Q22</t>
-        </is>
-      </c>
       <c r="G23">
         <v>1192</v>
       </c>
@@ -1864,11 +1754,6 @@
           <t>POSIXct, POSIXt</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Q23</t>
-        </is>
-      </c>
       <c r="G24">
         <v>1200</v>
       </c>
@@ -1914,11 +1799,6 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>numeric</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Q24</t>
         </is>
       </c>
       <c r="G25">

</xml_diff>

<commit_message>
sochealth gains a multiple-response block: five info_* items (sources of health information) drawn from a latent propensity with age, sex and education effects and a doctor/internet substitution, 36 respondents who skipped the question, 67 who chose nothing; the 24 existing columns are bit-identical; data documentation, vignette counts, codebook showcase and a data test updated
</commit_message>
<xml_diff>
--- a/pkgdown/assets/codebook/sochealth_codebook.xlsx
+++ b/pkgdown/assets/codebook/sochealth_codebook.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -610,7 +610,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>spicy 0.13.0.9000, R 4.6.1, 2026-10-09 19:18:00</t>
+          <t>spicy 0.14.0, R 4.6.1, 2026-10-18 12:10:33</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
@@ -1252,38 +1252,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_doctor</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Self-rated health</t>
+          <t>Doctor or other health professional</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>categorical (ordinal)</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ordered, factor</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="G14">
-        <v>1180</v>
+        <v>1164</v>
       </c>
       <c r="H14">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1292,50 +1292,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>wellbeing_score</t>
+          <t>info_pharmacist</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>WHO-5 wellbeing index (0-100)</t>
+          <t>Pharmacist</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="G15">
-        <v>1200</v>
+        <v>1164</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="K15">
-        <v>517</v>
-      </c>
-      <c r="M15">
-        <v>18.7</v>
-      </c>
-      <c r="N15">
-        <v>100</v>
-      </c>
-      <c r="O15" s="7">
-        <v>69.0405833333333</v>
-      </c>
-      <c r="P15" s="7">
-        <v>15.6203587559989</v>
-      </c>
-      <c r="Q15" s="7">
-        <v>70.25</v>
+        <v>2</v>
+      </c>
+      <c r="L15">
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1344,50 +1332,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bmi</t>
+          <t>info_internet</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Body mass index</t>
+          <t>Internet, websites or apps</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="G16">
-        <v>1188</v>
+        <v>1164</v>
       </c>
       <c r="H16">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="K16">
-        <v>177</v>
-      </c>
-      <c r="M16">
-        <v>16</v>
-      </c>
-      <c r="N16">
-        <v>38.9</v>
-      </c>
-      <c r="O16" s="8">
-        <v>25.9314814814815</v>
-      </c>
-      <c r="P16" s="8">
-        <v>3.72018590188177</v>
-      </c>
-      <c r="Q16" s="8">
-        <v>25.9</v>
+        <v>2</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1396,38 +1372,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>bmi_category</t>
+          <t>info_family</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BMI category</t>
+          <t>Family or friends</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>categorical (ordinal)</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ordered, factor</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="G17">
-        <v>1188</v>
+        <v>1164</v>
       </c>
       <c r="H17">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="I17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L17">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1436,38 +1412,38 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>institutional_trust</t>
+          <t>info_media</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Trust in institutions</t>
+          <t>Television, radio or newspapers</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>categorical (ordinal)</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ordered, factor</t>
+          <t>logical</t>
         </is>
       </c>
       <c r="G18">
-        <v>1200</v>
+        <v>1164</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L18">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1476,50 +1452,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>political_position</t>
+          <t>self_rated_health</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Political position (0 = left, 10 = right)</t>
+          <t>Self-rated health</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>categorical (ordinal)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>ordered, factor</t>
         </is>
       </c>
       <c r="G19">
-        <v>1185</v>
+        <v>1180</v>
       </c>
       <c r="H19">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>11</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>10</v>
-      </c>
-      <c r="O19" s="9">
-        <v>5.48016877637131</v>
-      </c>
-      <c r="P19" s="9">
-        <v>2.03387361047396</v>
-      </c>
-      <c r="Q19" s="9">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="L19">
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -1528,12 +1492,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>life_sat_health</t>
+          <t>wellbeing_score</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Satisfaction with health (1-5)</t>
+          <t>WHO-5 wellbeing index (0-100)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1543,35 +1507,35 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="G20">
-        <v>1192</v>
+        <v>1200</v>
       </c>
       <c r="H20">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>5</v>
+        <v>517</v>
       </c>
       <c r="M20">
-        <v>1</v>
+        <v>18.7</v>
       </c>
       <c r="N20">
-        <v>5</v>
-      </c>
-      <c r="O20" s="10">
-        <v>3.54865771812081</v>
-      </c>
-      <c r="P20" s="10">
-        <v>1.25008072026489</v>
-      </c>
-      <c r="Q20" s="10">
-        <v>4</v>
+        <v>100</v>
+      </c>
+      <c r="O20" s="7">
+        <v>69.0405833333333</v>
+      </c>
+      <c r="P20" s="7">
+        <v>15.6203587559989</v>
+      </c>
+      <c r="Q20" s="7">
+        <v>70.25</v>
       </c>
     </row>
     <row r="21">
@@ -1580,12 +1544,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>life_sat_work</t>
+          <t>bmi</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Satisfaction with work (1-5)</t>
+          <t>Body mass index</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1595,35 +1559,35 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="G21">
-        <v>1192</v>
+        <v>1188</v>
       </c>
       <c r="H21">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>177</v>
       </c>
       <c r="M21">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="N21">
-        <v>5</v>
-      </c>
-      <c r="O21" s="11">
-        <v>3.37835570469799</v>
-      </c>
-      <c r="P21" s="11">
-        <v>1.18497505958556</v>
-      </c>
-      <c r="Q21" s="11">
-        <v>3</v>
+        <v>38.9</v>
+      </c>
+      <c r="O21" s="8">
+        <v>25.9314814814815</v>
+      </c>
+      <c r="P21" s="8">
+        <v>3.72018590188177</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>25.9</v>
       </c>
     </row>
     <row r="22">
@@ -1632,50 +1596,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>life_sat_relationships</t>
+          <t>bmi_category</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Satisfaction with relationships (1-5)</t>
+          <t>BMI category</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>categorical (ordinal)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>ordered, factor</t>
         </is>
       </c>
       <c r="G22">
-        <v>1192</v>
+        <v>1188</v>
       </c>
       <c r="H22">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>5</v>
-      </c>
-      <c r="M22">
-        <v>1</v>
-      </c>
-      <c r="N22">
-        <v>5</v>
-      </c>
-      <c r="O22" s="12">
-        <v>3.7248322147651</v>
-      </c>
-      <c r="P22" s="12">
-        <v>1.09718553250181</v>
-      </c>
-      <c r="Q22" s="12">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="L22">
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -1684,49 +1636,37 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>life_sat_standard</t>
+          <t>institutional_trust</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Satisfaction with standard of living (1-5)</t>
+          <t>Trust in institutions</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>categorical (ordinal)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>ordered, factor</t>
         </is>
       </c>
       <c r="G23">
-        <v>1192</v>
+        <v>1200</v>
       </c>
       <c r="H23">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="K23">
-        <v>5</v>
-      </c>
-      <c r="M23">
-        <v>1</v>
-      </c>
-      <c r="N23">
-        <v>5</v>
-      </c>
-      <c r="O23" s="13">
-        <v>3.39681208053691</v>
-      </c>
-      <c r="P23" s="13">
-        <v>1.16025268893811</v>
-      </c>
-      <c r="Q23" s="13">
+        <v>4</v>
+      </c>
+      <c r="L23">
         <v>4</v>
       </c>
     </row>
@@ -1736,45 +1676,50 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>response_date</t>
+          <t>political_position</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Survey response date</t>
+          <t>Political position (0 = left, 10 = right)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>date-time</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>POSIXct, POSIXt</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="G24">
-        <v>1200</v>
+        <v>1185</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>1200</v>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>2024-09-02 08:30:40 Europe/Zurich</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>2024-11-30 03:26:27 Europe/Zurich</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>10</v>
+      </c>
+      <c r="O24" s="9">
+        <v>5.48016877637131</v>
+      </c>
+      <c r="P24" s="9">
+        <v>2.03387361047396</v>
+      </c>
+      <c r="Q24" s="9">
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -1783,49 +1728,304 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>life_sat_health</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Satisfaction with health (1-5)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="G25">
+        <v>1192</v>
+      </c>
+      <c r="H25">
+        <v>8</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
+      </c>
+      <c r="N25">
+        <v>5</v>
+      </c>
+      <c r="O25" s="10">
+        <v>3.54865771812081</v>
+      </c>
+      <c r="P25" s="10">
+        <v>1.25008072026489</v>
+      </c>
+      <c r="Q25" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>life_sat_work</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Satisfaction with work (1-5)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="G26">
+        <v>1192</v>
+      </c>
+      <c r="H26">
+        <v>8</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>5</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
+      </c>
+      <c r="N26">
+        <v>5</v>
+      </c>
+      <c r="O26" s="11">
+        <v>3.37835570469799</v>
+      </c>
+      <c r="P26" s="11">
+        <v>1.18497505958556</v>
+      </c>
+      <c r="Q26" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>life_sat_relationships</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Satisfaction with relationships (1-5)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="G27">
+        <v>1192</v>
+      </c>
+      <c r="H27">
+        <v>8</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>5</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
+      </c>
+      <c r="N27">
+        <v>5</v>
+      </c>
+      <c r="O27" s="12">
+        <v>3.7248322147651</v>
+      </c>
+      <c r="P27" s="12">
+        <v>1.09718553250181</v>
+      </c>
+      <c r="Q27" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>life_sat_standard</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Satisfaction with standard of living (1-5)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="G28">
+        <v>1192</v>
+      </c>
+      <c r="H28">
+        <v>8</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
+      </c>
+      <c r="N28">
+        <v>5</v>
+      </c>
+      <c r="O28" s="13">
+        <v>3.39681208053691</v>
+      </c>
+      <c r="P28" s="13">
+        <v>1.16025268893811</v>
+      </c>
+      <c r="Q28" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>response_date</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Survey response date</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>POSIXct, POSIXt</t>
+        </is>
+      </c>
+      <c r="G29">
+        <v>1200</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>1200</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>2024-09-02 08:30:40 Europe/Zurich</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>2024-11-30 03:26:27 Europe/Zurich</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Survey design weight</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="G25">
+      <c r="G30">
         <v>1200</v>
       </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="K25">
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="K30">
         <v>794</v>
       </c>
-      <c r="M25">
+      <c r="M30">
         <v>0.294</v>
       </c>
-      <c r="N25">
+      <c r="N30">
         <v>3.447</v>
       </c>
-      <c r="O25" s="14">
+      <c r="O30" s="14">
         <v>0.997061666666667</v>
       </c>
-      <c r="P25" s="14">
+      <c r="P30" s="14">
         <v>0.40625697754877</v>
       </c>
-      <c r="Q25" s="14">
+      <c r="Q30" s="14">
         <v>0.913</v>
       </c>
     </row>
@@ -1842,7 +2042,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="9.141"/>
@@ -2870,25 +3070,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_doctor</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E38" t="b">
         <v>0</v>
       </c>
       <c r="F38">
-        <v>61</v>
+        <v>443</v>
       </c>
       <c r="G38" s="4">
-        <v>5.08333333333333</v>
+        <v>36.9166666666667</v>
       </c>
       <c r="H38" s="4">
-        <v>5.16949152542373</v>
+        <v>38.0584192439863</v>
       </c>
     </row>
     <row r="39">
@@ -2897,25 +3097,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_doctor</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fair</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="E39" t="b">
         <v>0</v>
       </c>
       <c r="F39">
-        <v>266</v>
+        <v>721</v>
       </c>
       <c r="G39" s="4">
-        <v>22.1666666666667</v>
+        <v>60.0833333333333</v>
       </c>
       <c r="H39" s="4">
-        <v>22.5423728813559</v>
+        <v>61.9415807560137</v>
       </c>
     </row>
     <row r="40">
@@ -2924,167 +3124,165 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_doctor</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E40" t="b">
         <v>0</v>
       </c>
       <c r="F40">
-        <v>558</v>
+        <v>36</v>
       </c>
       <c r="G40" s="4">
-        <v>46.5</v>
-      </c>
-      <c r="H40" s="4">
-        <v>47.2881355932203</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H40" s="4"/>
     </row>
     <row r="41">
       <c r="A41">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_pharmacist</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Very good</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E41" t="b">
         <v>0</v>
       </c>
       <c r="F41">
-        <v>295</v>
+        <v>908</v>
       </c>
       <c r="G41" s="4">
-        <v>24.5833333333333</v>
+        <v>75.6666666666667</v>
       </c>
       <c r="H41" s="4">
-        <v>25</v>
+        <v>78.0068728522337</v>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>self_rated_health</t>
+          <t>info_pharmacist</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="E42" t="b">
         <v>0</v>
       </c>
       <c r="F42">
-        <v>20</v>
+        <v>256</v>
       </c>
       <c r="G42" s="4">
-        <v>1.66666666666667</v>
-      </c>
-      <c r="H42" s="4"/>
+        <v>21.3333333333333</v>
+      </c>
+      <c r="H42" s="4">
+        <v>21.9931271477663</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>bmi_category</t>
+          <t>info_pharmacist</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Normal weight</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E43" t="b">
         <v>0</v>
       </c>
       <c r="F43">
-        <v>465</v>
+        <v>36</v>
       </c>
       <c r="G43" s="4">
-        <v>38.75</v>
-      </c>
-      <c r="H43" s="4">
-        <v>39.1414141414141</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H43" s="4"/>
     </row>
     <row r="44">
       <c r="A44">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>bmi_category</t>
+          <t>info_internet</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Overweight</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E44" t="b">
         <v>0</v>
       </c>
       <c r="F44">
-        <v>569</v>
+        <v>641</v>
       </c>
       <c r="G44" s="4">
-        <v>47.4166666666667</v>
+        <v>53.4166666666667</v>
       </c>
       <c r="H44" s="4">
-        <v>47.8956228956229</v>
+        <v>55.0687285223368</v>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>bmi_category</t>
+          <t>info_internet</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Obesity</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="E45" t="b">
         <v>0</v>
       </c>
       <c r="F45">
-        <v>154</v>
+        <v>523</v>
       </c>
       <c r="G45" s="4">
-        <v>12.8333333333333</v>
+        <v>43.5833333333333</v>
       </c>
       <c r="H45" s="4">
-        <v>12.962962962963</v>
+        <v>44.9312714776632</v>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>bmi_category</t>
+          <t>info_internet</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3096,93 +3294,91 @@
         <v>0</v>
       </c>
       <c r="F46">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="G46" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H46" s="4"/>
     </row>
     <row r="47">
       <c r="A47">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>institutional_trust</t>
+          <t>info_family</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Very low</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E47" t="b">
         <v>0</v>
       </c>
       <c r="F47">
-        <v>366</v>
+        <v>804</v>
       </c>
       <c r="G47" s="4">
-        <v>30.5</v>
+        <v>67</v>
       </c>
       <c r="H47" s="4">
-        <v>30.5</v>
+        <v>69.0721649484536</v>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>institutional_trust</t>
+          <t>info_family</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="E48" t="b">
         <v>0</v>
       </c>
       <c r="F48">
-        <v>472</v>
+        <v>360</v>
       </c>
       <c r="G48" s="4">
-        <v>39.3333333333333</v>
+        <v>30</v>
       </c>
       <c r="H48" s="4">
-        <v>39.3333333333333</v>
+        <v>30.9278350515464</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>institutional_trust</t>
+          <t>info_family</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E49" t="b">
         <v>0</v>
       </c>
       <c r="F49">
-        <v>234</v>
+        <v>36</v>
       </c>
       <c r="G49" s="4">
-        <v>19.5</v>
-      </c>
-      <c r="H49" s="4">
-        <v>19.5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H49" s="4"/>
     </row>
     <row r="50">
       <c r="A50">
@@ -3190,24 +3386,423 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>info_media</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>1023</v>
+      </c>
+      <c r="G50" s="4">
+        <v>85.25</v>
+      </c>
+      <c r="H50" s="4">
+        <v>87.8865979381443</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>17</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>info_media</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>141</v>
+      </c>
+      <c r="G51" s="4">
+        <v>11.75</v>
+      </c>
+      <c r="H51" s="4">
+        <v>12.1134020618557</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>17</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>info_media</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E52" t="b">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>36</v>
+      </c>
+      <c r="G52" s="4">
+        <v>3</v>
+      </c>
+      <c r="H52" s="4"/>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>18</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>self_rated_health</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="E53" t="b">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>61</v>
+      </c>
+      <c r="G53" s="4">
+        <v>5.08333333333333</v>
+      </c>
+      <c r="H53" s="4">
+        <v>5.16949152542373</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>18</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>self_rated_health</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Fair</t>
+        </is>
+      </c>
+      <c r="E54" t="b">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>266</v>
+      </c>
+      <c r="G54" s="4">
+        <v>22.1666666666667</v>
+      </c>
+      <c r="H54" s="4">
+        <v>22.5423728813559</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>18</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>self_rated_health</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="E55" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>558</v>
+      </c>
+      <c r="G55" s="4">
+        <v>46.5</v>
+      </c>
+      <c r="H55" s="4">
+        <v>47.2881355932203</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>18</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>self_rated_health</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Very good</t>
+        </is>
+      </c>
+      <c r="E56" t="b">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>295</v>
+      </c>
+      <c r="G56" s="4">
+        <v>24.5833333333333</v>
+      </c>
+      <c r="H56" s="4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>18</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>self_rated_health</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E57" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>20</v>
+      </c>
+      <c r="G57" s="4">
+        <v>1.66666666666667</v>
+      </c>
+      <c r="H57" s="4"/>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>21</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>bmi_category</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Normal weight</t>
+        </is>
+      </c>
+      <c r="E58" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>465</v>
+      </c>
+      <c r="G58" s="4">
+        <v>38.75</v>
+      </c>
+      <c r="H58" s="4">
+        <v>39.1414141414141</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>21</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>bmi_category</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Overweight</t>
+        </is>
+      </c>
+      <c r="E59" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>569</v>
+      </c>
+      <c r="G59" s="4">
+        <v>47.4166666666667</v>
+      </c>
+      <c r="H59" s="4">
+        <v>47.8956228956229</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>21</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>bmi_category</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Obesity</t>
+        </is>
+      </c>
+      <c r="E60" t="b">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>154</v>
+      </c>
+      <c r="G60" s="4">
+        <v>12.8333333333333</v>
+      </c>
+      <c r="H60" s="4">
+        <v>12.962962962963</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>21</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>bmi_category</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="E61" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>12</v>
+      </c>
+      <c r="G61" s="4">
+        <v>1</v>
+      </c>
+      <c r="H61" s="4"/>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>22</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>institutional_trust</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Very low</t>
+        </is>
+      </c>
+      <c r="E62" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>366</v>
+      </c>
+      <c r="G62" s="4">
+        <v>30.5</v>
+      </c>
+      <c r="H62" s="4">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>22</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>institutional_trust</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E63" t="b">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>472</v>
+      </c>
+      <c r="G63" s="4">
+        <v>39.3333333333333</v>
+      </c>
+      <c r="H63" s="4">
+        <v>39.3333333333333</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>22</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>institutional_trust</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E64" t="b">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>234</v>
+      </c>
+      <c r="G64" s="4">
+        <v>19.5</v>
+      </c>
+      <c r="H64" s="4">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>22</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>institutional_trust</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
         <is>
           <t>Very high</t>
         </is>
       </c>
-      <c r="E50" t="b">
-        <v>0</v>
-      </c>
-      <c r="F50">
+      <c r="E65" t="b">
+        <v>0</v>
+      </c>
+      <c r="F65">
         <v>128</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G65" s="4">
         <v>10.6666666666667</v>
       </c>
-      <c r="H50" s="4">
+      <c r="H65" s="4">
         <v>10.6666666666667</v>
       </c>
     </row>

</xml_diff>